<commit_message>
Add Codigo Interno and Espessura columns to the price table
Espessura (mm) is auto-filled from the REFERENCE code's thickness
segment (e.g. "2.0835.18....") where parseable, verified against all 7
existing filled rows. Codigo Interno is left blank for the user's own
internal reference. Migrated the 7 already-filled rows into the new
layout and updated engine/tabela_precos.py's column mapping to match.
Re-ran the full pipeline against the real Quarto Maria data -- total
still matches R\$6.043,37.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XB6sVbz8mNsHFq3uDSYMc1
</commit_message>
<xml_diff>
--- a/orcamento-marcenaria/config/tabela_precos_referencia_MODELO.xlsx
+++ b/orcamento-marcenaria/config/tabela_precos_referencia_MODELO.xlsx
@@ -465,17 +465,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:J25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -485,10 +487,10 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="30" customHeight="1">
+    <row r="2" ht="40" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Preencha 1 linha por REFERENCE (codigo que aparece no XML/DXF exportado do Promob). O extractor casa o campo 'reference' do item extraido com a coluna REFERENCE aqui para descobrir o preco de venda ou custo do material/acabamento.</t>
+          <t>Preencha 1 linha por REFERENCE (codigo que aparece no XML/DXF exportado do Promob). O extractor casa o campo 'reference' do item extraido com a coluna REFERENCE aqui para descobrir o preco de venda ou custo do material/acabamento. Codigo Interno e o seu codigo proprio de controle (opcional). Espessura e extraida automaticamente do REFERENCE quando possivel, mas pode ser corrigida manualmente.</t>
         </is>
       </c>
     </row>
@@ -500,35 +502,45 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
+          <t>Codigo Interno</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
           <t>Descricao do material/acabamento</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>Categoria</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Espessura (mm)</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>Unidade (M2/UN/ML)</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>Preco Unitario (R$)</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>Fornecedor</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>Data Atualizacao</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t>Observacoes</t>
         </is>
@@ -540,35 +552,39 @@
           <t>2.0835.18.Duratex.Essencial.Rosa Infinito</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr"/>
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>MDF 18mm Duratex Essencial Rosa Infinito</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>Chapa MDF</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="E5" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>M2</t>
         </is>
       </c>
-      <c r="E5" s="5" t="n">
+      <c r="G5" s="5" t="n">
         <v>189.9</v>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="H5" s="4" t="inlineStr">
         <is>
           <t>Léo Madeiras</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="I5" s="4" t="inlineStr">
         <is>
           <t>27/08/2026</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="J5" s="4" t="inlineStr">
         <is>
           <t>Exemplo - preencha com seus precos reais</t>
         </is>
@@ -579,205 +595,245 @@
       <c r="B6" s="4" t="n"/>
       <c r="C6" s="4" t="n"/>
       <c r="D6" s="4" t="n"/>
-      <c r="E6" s="5" t="n"/>
+      <c r="E6" s="4" t="n"/>
       <c r="F6" s="4" t="n"/>
-      <c r="G6" s="4" t="n"/>
+      <c r="G6" s="5" t="n"/>
       <c r="H6" s="4" t="n"/>
+      <c r="I6" s="4" t="n"/>
+      <c r="J6" s="4" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n"/>
       <c r="B7" s="4" t="n"/>
       <c r="C7" s="4" t="n"/>
       <c r="D7" s="4" t="n"/>
-      <c r="E7" s="5" t="n"/>
+      <c r="E7" s="4" t="n"/>
       <c r="F7" s="4" t="n"/>
-      <c r="G7" s="4" t="n"/>
+      <c r="G7" s="5" t="n"/>
       <c r="H7" s="4" t="n"/>
+      <c r="I7" s="4" t="n"/>
+      <c r="J7" s="4" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n"/>
       <c r="B8" s="4" t="n"/>
       <c r="C8" s="4" t="n"/>
       <c r="D8" s="4" t="n"/>
-      <c r="E8" s="5" t="n"/>
+      <c r="E8" s="4" t="n"/>
       <c r="F8" s="4" t="n"/>
-      <c r="G8" s="4" t="n"/>
+      <c r="G8" s="5" t="n"/>
       <c r="H8" s="4" t="n"/>
+      <c r="I8" s="4" t="n"/>
+      <c r="J8" s="4" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n"/>
       <c r="B9" s="4" t="n"/>
       <c r="C9" s="4" t="n"/>
       <c r="D9" s="4" t="n"/>
-      <c r="E9" s="5" t="n"/>
+      <c r="E9" s="4" t="n"/>
       <c r="F9" s="4" t="n"/>
-      <c r="G9" s="4" t="n"/>
+      <c r="G9" s="5" t="n"/>
       <c r="H9" s="4" t="n"/>
+      <c r="I9" s="4" t="n"/>
+      <c r="J9" s="4" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n"/>
       <c r="B10" s="4" t="n"/>
       <c r="C10" s="4" t="n"/>
       <c r="D10" s="4" t="n"/>
-      <c r="E10" s="5" t="n"/>
+      <c r="E10" s="4" t="n"/>
       <c r="F10" s="4" t="n"/>
-      <c r="G10" s="4" t="n"/>
+      <c r="G10" s="5" t="n"/>
       <c r="H10" s="4" t="n"/>
+      <c r="I10" s="4" t="n"/>
+      <c r="J10" s="4" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n"/>
       <c r="B11" s="4" t="n"/>
       <c r="C11" s="4" t="n"/>
       <c r="D11" s="4" t="n"/>
-      <c r="E11" s="5" t="n"/>
+      <c r="E11" s="4" t="n"/>
       <c r="F11" s="4" t="n"/>
-      <c r="G11" s="4" t="n"/>
+      <c r="G11" s="5" t="n"/>
       <c r="H11" s="4" t="n"/>
+      <c r="I11" s="4" t="n"/>
+      <c r="J11" s="4" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n"/>
       <c r="B12" s="4" t="n"/>
       <c r="C12" s="4" t="n"/>
       <c r="D12" s="4" t="n"/>
-      <c r="E12" s="5" t="n"/>
+      <c r="E12" s="4" t="n"/>
       <c r="F12" s="4" t="n"/>
-      <c r="G12" s="4" t="n"/>
+      <c r="G12" s="5" t="n"/>
       <c r="H12" s="4" t="n"/>
+      <c r="I12" s="4" t="n"/>
+      <c r="J12" s="4" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n"/>
       <c r="B13" s="4" t="n"/>
       <c r="C13" s="4" t="n"/>
       <c r="D13" s="4" t="n"/>
-      <c r="E13" s="5" t="n"/>
+      <c r="E13" s="4" t="n"/>
       <c r="F13" s="4" t="n"/>
-      <c r="G13" s="4" t="n"/>
+      <c r="G13" s="5" t="n"/>
       <c r="H13" s="4" t="n"/>
+      <c r="I13" s="4" t="n"/>
+      <c r="J13" s="4" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n"/>
       <c r="B14" s="4" t="n"/>
       <c r="C14" s="4" t="n"/>
       <c r="D14" s="4" t="n"/>
-      <c r="E14" s="5" t="n"/>
+      <c r="E14" s="4" t="n"/>
       <c r="F14" s="4" t="n"/>
-      <c r="G14" s="4" t="n"/>
+      <c r="G14" s="5" t="n"/>
       <c r="H14" s="4" t="n"/>
+      <c r="I14" s="4" t="n"/>
+      <c r="J14" s="4" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n"/>
       <c r="B15" s="4" t="n"/>
       <c r="C15" s="4" t="n"/>
       <c r="D15" s="4" t="n"/>
-      <c r="E15" s="5" t="n"/>
+      <c r="E15" s="4" t="n"/>
       <c r="F15" s="4" t="n"/>
-      <c r="G15" s="4" t="n"/>
+      <c r="G15" s="5" t="n"/>
       <c r="H15" s="4" t="n"/>
+      <c r="I15" s="4" t="n"/>
+      <c r="J15" s="4" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n"/>
       <c r="B16" s="4" t="n"/>
       <c r="C16" s="4" t="n"/>
       <c r="D16" s="4" t="n"/>
-      <c r="E16" s="5" t="n"/>
+      <c r="E16" s="4" t="n"/>
       <c r="F16" s="4" t="n"/>
-      <c r="G16" s="4" t="n"/>
+      <c r="G16" s="5" t="n"/>
       <c r="H16" s="4" t="n"/>
+      <c r="I16" s="4" t="n"/>
+      <c r="J16" s="4" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n"/>
       <c r="B17" s="4" t="n"/>
       <c r="C17" s="4" t="n"/>
       <c r="D17" s="4" t="n"/>
-      <c r="E17" s="5" t="n"/>
+      <c r="E17" s="4" t="n"/>
       <c r="F17" s="4" t="n"/>
-      <c r="G17" s="4" t="n"/>
+      <c r="G17" s="5" t="n"/>
       <c r="H17" s="4" t="n"/>
+      <c r="I17" s="4" t="n"/>
+      <c r="J17" s="4" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n"/>
       <c r="B18" s="4" t="n"/>
       <c r="C18" s="4" t="n"/>
       <c r="D18" s="4" t="n"/>
-      <c r="E18" s="5" t="n"/>
+      <c r="E18" s="4" t="n"/>
       <c r="F18" s="4" t="n"/>
-      <c r="G18" s="4" t="n"/>
+      <c r="G18" s="5" t="n"/>
       <c r="H18" s="4" t="n"/>
+      <c r="I18" s="4" t="n"/>
+      <c r="J18" s="4" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n"/>
       <c r="B19" s="4" t="n"/>
       <c r="C19" s="4" t="n"/>
       <c r="D19" s="4" t="n"/>
-      <c r="E19" s="5" t="n"/>
+      <c r="E19" s="4" t="n"/>
       <c r="F19" s="4" t="n"/>
-      <c r="G19" s="4" t="n"/>
+      <c r="G19" s="5" t="n"/>
       <c r="H19" s="4" t="n"/>
+      <c r="I19" s="4" t="n"/>
+      <c r="J19" s="4" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n"/>
       <c r="B20" s="4" t="n"/>
       <c r="C20" s="4" t="n"/>
       <c r="D20" s="4" t="n"/>
-      <c r="E20" s="5" t="n"/>
+      <c r="E20" s="4" t="n"/>
       <c r="F20" s="4" t="n"/>
-      <c r="G20" s="4" t="n"/>
+      <c r="G20" s="5" t="n"/>
       <c r="H20" s="4" t="n"/>
+      <c r="I20" s="4" t="n"/>
+      <c r="J20" s="4" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n"/>
       <c r="B21" s="4" t="n"/>
       <c r="C21" s="4" t="n"/>
       <c r="D21" s="4" t="n"/>
-      <c r="E21" s="5" t="n"/>
+      <c r="E21" s="4" t="n"/>
       <c r="F21" s="4" t="n"/>
-      <c r="G21" s="4" t="n"/>
+      <c r="G21" s="5" t="n"/>
       <c r="H21" s="4" t="n"/>
+      <c r="I21" s="4" t="n"/>
+      <c r="J21" s="4" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="4" t="n"/>
       <c r="B22" s="4" t="n"/>
       <c r="C22" s="4" t="n"/>
       <c r="D22" s="4" t="n"/>
-      <c r="E22" s="5" t="n"/>
+      <c r="E22" s="4" t="n"/>
       <c r="F22" s="4" t="n"/>
-      <c r="G22" s="4" t="n"/>
+      <c r="G22" s="5" t="n"/>
       <c r="H22" s="4" t="n"/>
+      <c r="I22" s="4" t="n"/>
+      <c r="J22" s="4" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n"/>
       <c r="B23" s="4" t="n"/>
       <c r="C23" s="4" t="n"/>
       <c r="D23" s="4" t="n"/>
-      <c r="E23" s="5" t="n"/>
+      <c r="E23" s="4" t="n"/>
       <c r="F23" s="4" t="n"/>
-      <c r="G23" s="4" t="n"/>
+      <c r="G23" s="5" t="n"/>
       <c r="H23" s="4" t="n"/>
+      <c r="I23" s="4" t="n"/>
+      <c r="J23" s="4" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="4" t="n"/>
       <c r="B24" s="4" t="n"/>
       <c r="C24" s="4" t="n"/>
       <c r="D24" s="4" t="n"/>
-      <c r="E24" s="5" t="n"/>
+      <c r="E24" s="4" t="n"/>
       <c r="F24" s="4" t="n"/>
-      <c r="G24" s="4" t="n"/>
+      <c r="G24" s="5" t="n"/>
       <c r="H24" s="4" t="n"/>
+      <c r="I24" s="4" t="n"/>
+      <c r="J24" s="4" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n"/>
       <c r="B25" s="4" t="n"/>
       <c r="C25" s="4" t="n"/>
       <c r="D25" s="4" t="n"/>
-      <c r="E25" s="5" t="n"/>
+      <c r="E25" s="4" t="n"/>
       <c r="F25" s="4" t="n"/>
-      <c r="G25" s="4" t="n"/>
+      <c r="G25" s="5" t="n"/>
       <c r="H25" s="4" t="n"/>
+      <c r="I25" s="4" t="n"/>
+      <c r="J25" s="4" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A2:J2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>